<commit_message>
update: 2026-04-17 | +1 new, +0 updates, +0 promotions | Evive Biotech Ryzneuta® Italy/Poland commercial rights to Molteni
- NEW (Actionable): Evive Biotech (亿一生物) → Molteni Farmaceutici
  efbemalenograstim alfa (G-CSF Fc-fusion), Approved US/CN/EU
  Italy + Poland commercial rights; financials undisclosed
- company_names.md: added 亿一生物 → Evive Biotech (Private, subsidiary of Yifan Pharma SH:002019)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracker/bd_tracker.xlsx
+++ b/tracker/bd_tracker.xlsx
@@ -669,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="10.2"/>
   <cols>
     <col width="23.6640625" customWidth="1" style="11" min="1" max="1"/>
@@ -765,101 +765,101 @@
       </c>
     </row>
     <row r="2" ht="26.1" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
-        <is>
-          <t>Foresee Pharma (逸达生物)</t>
-        </is>
-      </c>
-      <c r="B2" s="15" t="inlineStr">
-        <is>
-          <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="C2" s="15" t="inlineStr">
-        <is>
-          <t>Primevera Therapeutics</t>
-        </is>
-      </c>
-      <c r="D2" s="15" t="inlineStr">
-        <is>
-          <t>aderamastat (MMP12 | MMP12inh.)</t>
-        </is>
-      </c>
-      <c r="E2" s="15" t="inlineStr">
-        <is>
-          <t>Small Mol.</t>
-        </is>
-      </c>
-      <c r="F2" s="24" t="inlineStr">
-        <is>
-          <t>Ph2/3</t>
-        </is>
-      </c>
-      <c r="G2" s="16" t="inlineStr">
-        <is>
-          <t>Preclnl</t>
-        </is>
-      </c>
-      <c r="H2" s="16" t="inlineStr">
-        <is>
-          <t>Ph2</t>
-        </is>
-      </c>
-      <c r="I2" s="16" t="inlineStr">
-        <is>
-          <t>Preclnl</t>
-        </is>
-      </c>
-      <c r="J2" s="16" t="inlineStr">
-        <is>
-          <t>$584m</t>
-        </is>
-      </c>
-      <c r="K2" s="16" t="inlineStr">
-        <is>
-          <t>$10m</t>
-        </is>
-      </c>
-      <c r="L2" s="15" t="inlineStr">
-        <is>
-          <t>COVID-19; ARDS; COPD</t>
-        </is>
-      </c>
-      <c r="M2" s="15" t="inlineStr">
-        <is>
-          <t>All rights: Global</t>
-        </is>
-      </c>
-      <c r="N2" s="15" t="inlineStr">
-        <is>
-          <t>2026-01-08</t>
-        </is>
-      </c>
-      <c r="O2" s="17" t="inlineStr">
-        <is>
-          <t>Potential FIC. Global all rights out-licensed. TW-listed, respiratory niche (COPD/asthma). MMP12 is a differentiated target but commercial path is long. Small deal ($585M total, $10M upfront).</t>
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Evive Biotech (亿一生物)</t>
+        </is>
+      </c>
+      <c r="B2" s="27" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C2" s="27" t="inlineStr">
+        <is>
+          <t>Molteni Farmaceutici</t>
+        </is>
+      </c>
+      <c r="D2" s="27" t="inlineStr">
+        <is>
+          <t>efbemalenograstim alfa (G-CSF)</t>
+        </is>
+      </c>
+      <c r="E2" s="27" t="inlineStr">
+        <is>
+          <t>Fusion Protein</t>
+        </is>
+      </c>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="G2" s="29" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H2" s="29" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="I2" s="29" t="inlineStr">
+        <is>
+          <t>Preclnl</t>
+        </is>
+      </c>
+      <c r="J2" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K2" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L2" s="27" t="inlineStr">
+        <is>
+          <t>CIN; Febrile Neutropenia</t>
+        </is>
+      </c>
+      <c r="M2" s="27" t="inlineStr">
+        <is>
+          <t>Commercial rights: Italy; Poland</t>
+        </is>
+      </c>
+      <c r="N2" s="27" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="O2" s="30" t="inlineStr">
+        <is>
+          <t>Approved G-CSF Fc-fusion (Ryzneuta®) — US FDA 2023, CN/EU approved. Italy + Poland commercial rights to Molteni; financials undisclosed. Narrow geographic carve-out; Evive is private subsidiary of listed Yifan Pharma (SH:002019), limited royalty scale from small territories.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="26.1" customHeight="1">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>Hansoh Pharma (翰森制药)</t>
+          <t>Foresee Pharma (逸达生物)</t>
         </is>
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="C3" s="15" t="inlineStr">
         <is>
-          <t>Glenmark Specialty</t>
+          <t>Primevera Therapeutics</t>
         </is>
       </c>
       <c r="D3" s="15" t="inlineStr">
         <is>
-          <t>aumolertinib (EGFR T790M | EGFR T790Minh.)</t>
+          <t>aderamastat (MMP12 | MMP12inh.)</t>
         </is>
       </c>
       <c r="E3" s="15" t="inlineStr">
@@ -869,17 +869,17 @@
       </c>
       <c r="F3" s="24" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Ph2/3</t>
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Ph2</t>
         </is>
       </c>
       <c r="I3" s="16" t="inlineStr">
@@ -889,39 +889,39 @@
       </c>
       <c r="J3" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$584m</t>
         </is>
       </c>
       <c r="K3" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$10m</t>
         </is>
       </c>
       <c r="L3" s="15" t="inlineStr">
         <is>
-          <t>non-sq NSCLC; Lung Ca; Solid tumors</t>
+          <t>COVID-19; ARDS; COPD</t>
         </is>
       </c>
       <c r="M3" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: ROW | Commercial rights: ROW</t>
+          <t>All rights: Global</t>
         </is>
       </c>
       <c r="N3" s="15" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="O3" s="17" t="inlineStr">
         <is>
-          <t>Ex-CN R&amp;D + commercial to Glenmark for emerging markets. 3rd-gen EGFR TKI approved in CN with growing revenue. Hansoh is profitable and well-capitalized, unlikely to need royalty financing. Deal scope limited to emerging markets.</t>
+          <t>Potential FIC. Global all rights out-licensed. TW-listed, respiratory niche (COPD/asthma). MMP12 is a differentiated target but commercial path is long. Small deal ($585M total, $10M upfront).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="26.1" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>Innovent Biologics (信达生物)</t>
+          <t>Hansoh Pharma (翰森制药)</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
@@ -931,17 +931,17 @@
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>Takeda Pharmaceuticals</t>
+          <t>Glenmark Specialty</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>IBI363 (IL-2; PD1 | IL-Ab-fusion)</t>
+          <t>aumolertinib (EGFR T790M | EGFR T790Minh.)</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>Fusion Protein</t>
+          <t>Small Mol.</t>
         </is>
       </c>
       <c r="F4" s="24" t="inlineStr">
@@ -951,12 +951,12 @@
       </c>
       <c r="G4" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="H4" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="I4" s="16" t="inlineStr">
@@ -966,32 +966,32 @@
       </c>
       <c r="J4" s="16" t="inlineStr">
         <is>
-          <t>$11.4bn</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K4" s="16" t="inlineStr">
         <is>
-          <t>$1.2bn</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L4" s="15" t="inlineStr">
         <is>
-          <t>sq NSCLC; Melanoma; Pancreatic Ca</t>
+          <t>non-sq NSCLC; Lung Ca; Solid tumors</t>
         </is>
       </c>
       <c r="M4" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: Global | Mfg rights: US;EU;JP;ROW | Commercial rights: US;EU;JP;ROW</t>
+          <t>R&amp;D rights: ROW | Commercial rights: ROW</t>
         </is>
       </c>
       <c r="N4" s="15" t="inlineStr">
         <is>
-          <t>2025-10-21</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="O4" s="17" t="inlineStr">
         <is>
-          <t>Potential FIC. Global R&amp;D + ex-CN commercial rights to Takeda. IL-2×PD1 fusion protein, $11.4bn mega-deal with $1.2bn upfront, Takeda's largest BD deal ever. Innovent retains CN rights but faces heavy R&amp;D burn across broad pipeline. Future royalty stream could be very large if approved. Worth exploring whether Innovent would monetize a portion of retained economics.</t>
+          <t>Ex-CN R&amp;D + commercial to Glenmark for emerging markets. 3rd-gen EGFR TKI approved in CN with growing revenue. Hansoh is profitable and well-capitalized, unlikely to need royalty financing. Deal scope limited to emerging markets.</t>
         </is>
       </c>
     </row>
@@ -1008,22 +1008,22 @@
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>Takeda Pharmaceuticals(Top20 MNC)</t>
+          <t>Takeda Pharmaceuticals</t>
         </is>
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>IBI343 (CLDN18.2 | anti-CLDN18.2ADC)</t>
+          <t>IBI363 (IL-2; PD1 | IL-Ab-fusion)</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>ADC</t>
+          <t>Fusion Protein</t>
         </is>
       </c>
       <c r="F5" s="24" t="inlineStr">
         <is>
-          <t>Ph1</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="I5" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="J5" s="16" t="inlineStr">
@@ -1053,12 +1053,12 @@
       </c>
       <c r="L5" s="15" t="inlineStr">
         <is>
-          <t>Gastric Ca; PDAC; Solid tumors</t>
+          <t>sq NSCLC; Melanoma; Pancreatic Ca</t>
         </is>
       </c>
       <c r="M5" s="15" t="inlineStr">
         <is>
-          <t>All rights: US;EU;JP;ROW</t>
+          <t>R&amp;D rights: Global | Mfg rights: US;EU;JP;ROW | Commercial rights: US;EU;JP;ROW</t>
         </is>
       </c>
       <c r="N5" s="15" t="inlineStr">
@@ -1068,14 +1068,14 @@
       </c>
       <c r="O5" s="17" t="inlineStr">
         <is>
-          <t>Potential FIC. Ex-CN all rights to Takeda. CLDN18.2 ADC for gastric/pancreatic, US Ph1, CN Ph3, JP Ph3. Part of $11.4bn mega-deal. Innovent retains CN rights, could explore royalty financing on Takeda ex-CN stream to fund CN development and broader pipeline.</t>
+          <t>Potential FIC. Global R&amp;D + ex-CN commercial rights to Takeda. IL-2×PD1 fusion protein, $11.4bn mega-deal with $1.2bn upfront, Takeda's largest BD deal ever. Innovent retains CN rights but faces heavy R&amp;D burn across broad pipeline. Future royalty stream could be very large if approved. Worth exploring whether Innovent would monetize a portion of retained economics.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="26.1" customHeight="1">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>HaiHe Biopharma (海和药物)</t>
+          <t>Innovent Biologics (信达生物)</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
@@ -1085,17 +1085,17 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Taiho Pharmaceutical</t>
+          <t>Takeda Pharmaceuticals(Top20 MNC)</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>inavolisib (PI3Kα | PI3Kαinh.)</t>
+          <t>IBI343 (CLDN18.2 | anti-CLDN18.2ADC)</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>Small Mol.</t>
+          <t>ADC</t>
         </is>
       </c>
       <c r="F6" s="24" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>Ph2</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="H6" s="16" t="inlineStr">
@@ -1115,44 +1115,44 @@
       </c>
       <c r="I6" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="J6" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$11.4bn</t>
         </is>
       </c>
       <c r="K6" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$1.2bn</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
         <is>
-          <t>Vascular Malformation; GEJ Ca; Endometrial Ca</t>
+          <t>Gastric Ca; PDAC; Solid tumors</t>
         </is>
       </c>
       <c r="M6" s="15" t="inlineStr">
         <is>
-          <t>All rights: JP</t>
+          <t>All rights: US;EU;JP;ROW</t>
         </is>
       </c>
       <c r="N6" s="15" t="inlineStr">
         <is>
-          <t>2025-10-16</t>
+          <t>2025-10-21</t>
         </is>
       </c>
       <c r="O6" s="17" t="inlineStr">
         <is>
-          <t>JP-only rights. (all rights). Taiho Japan-only deal; limited geography</t>
+          <t>Potential FIC. Ex-CN all rights to Takeda. CLDN18.2 ADC for gastric/pancreatic, US Ph1, CN Ph3, JP Ph3. Part of $11.4bn mega-deal. Innovent retains CN rights, could explore royalty financing on Takeda ex-CN stream to fund CN development and broader pipeline.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="26.1" customHeight="1">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>InnoCare Pharma (诺诚健华)</t>
+          <t>HaiHe Biopharma (海和药物)</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
@@ -1162,12 +1162,12 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>Zenas BioPharma</t>
+          <t>Taiho Pharmaceutical</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>orelabrutinib (BTK | BTKinh.)</t>
+          <t>inavolisib (PI3Kα | PI3Kαinh.)</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
@@ -1177,74 +1177,74 @@
       </c>
       <c r="F7" s="24" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Ph1</t>
         </is>
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
+          <t>Ph2</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Preclnl</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
-        <is>
-          <t>Ph2</t>
-        </is>
-      </c>
-      <c r="I7" s="16" t="inlineStr">
-        <is>
-          <t>Preclnl</t>
-        </is>
-      </c>
       <c r="J7" s="16" t="inlineStr">
         <is>
-          <t>$2.1bn</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K7" s="16" t="inlineStr">
         <is>
-          <t>$60m</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L7" s="15" t="inlineStr">
         <is>
-          <t>DLBCL; Autoimmune Disease; WM</t>
+          <t>Vascular Malformation; GEJ Ca; Endometrial Ca</t>
         </is>
       </c>
       <c r="M7" s="15" t="inlineStr">
         <is>
-          <t>All rights: US;EU;JP;ROW | All rights: Global</t>
+          <t>All rights: JP</t>
         </is>
       </c>
       <c r="N7" s="15" t="inlineStr">
         <is>
-          <t>2025-10-07</t>
+          <t>2025-10-16</t>
         </is>
       </c>
       <c r="O7" s="17" t="inlineStr">
         <is>
-          <t>Ex-CN all rights to Zenas. BTK inhibitor approved in CN, US Ph3 for autoimmune indications, large TAM in ITP/SLE. $60M upfront on $2.1bn total is back-loaded. InnoCare is HK-listed with moderate cash, heavy autoimmune expansion spend. Royalty monetization could help fund CN commercial build-out.</t>
+          <t>JP-only rights. (all rights). Taiho Japan-only deal; limited geography</t>
         </is>
       </c>
     </row>
     <row r="8" ht="26.1" customHeight="1">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>Hanmi Pharmaceuticals</t>
+          <t>InnoCare Pharma (诺诚健华)</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Korea</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Gilead Sciences</t>
+          <t>Zenas BioPharma</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>encequidar (P-gp | P-gpinh.)</t>
+          <t>orelabrutinib (BTK | BTKinh.)</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
@@ -1254,17 +1254,17 @@
       </c>
       <c r="F8" s="24" t="inlineStr">
         <is>
-          <t>NDA Filed</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="G8" s="16" t="inlineStr">
         <is>
-          <t>Ph1</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="H8" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Ph2</t>
         </is>
       </c>
       <c r="I8" s="16" t="inlineStr">
@@ -1274,74 +1274,74 @@
       </c>
       <c r="J8" s="16" t="inlineStr">
         <is>
-          <t>$34m</t>
+          <t>$2.1bn</t>
         </is>
       </c>
       <c r="K8" s="16" t="inlineStr">
         <is>
-          <t>$2m</t>
+          <t>$60m</t>
         </is>
       </c>
       <c r="L8" s="15" t="inlineStr">
         <is>
-          <t>HER2+ Breast Ca; Gastric Ca; angiosarcoma</t>
+          <t>DLBCL; Autoimmune Disease; WM</t>
         </is>
       </c>
       <c r="M8" s="15" t="inlineStr">
         <is>
-          <t>All rights: Global</t>
+          <t>All rights: US;EU;JP;ROW | All rights: Global</t>
         </is>
       </c>
       <c r="N8" s="15" t="inlineStr">
         <is>
-          <t>2025-09-29</t>
+          <t>2025-10-07</t>
         </is>
       </c>
       <c r="O8" s="17" t="inlineStr">
         <is>
-          <t>Global all rights to Gilead. US NDA filed. Hanmi is large KR pharma, generally well-capitalized. Small deal ($34.5M).</t>
+          <t>Ex-CN all rights to Zenas. BTK inhibitor approved in CN, US Ph3 for autoimmune indications, large TAM in ITP/SLE. $60M upfront on $2.1bn total is back-loaded. InnoCare is HK-listed with moderate cash, heavy autoimmune expansion spend. Royalty monetization could help fund CN commercial build-out.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="26.1" customHeight="1">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>CStone Pharmaceuticals (基石药业)</t>
+          <t>Hanmi Pharmaceuticals</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Korea</t>
         </is>
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>Istituto Gentili</t>
+          <t>Gilead Sciences</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>sugemalimab (PDL1 | mAb)</t>
+          <t>encequidar (P-gp | P-gpinh.)</t>
         </is>
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>mAb</t>
+          <t>Small Mol.</t>
         </is>
       </c>
       <c r="F9" s="24" t="inlineStr">
         <is>
+          <t>NDA Filed</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
           <t>Ph1</t>
         </is>
       </c>
-      <c r="G9" s="16" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
       <c r="H9" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="I9" s="16" t="inlineStr">
@@ -1351,39 +1351,39 @@
       </c>
       <c r="J9" s="16" t="inlineStr">
         <is>
-          <t>$192m</t>
+          <t>$34m</t>
         </is>
       </c>
       <c r="K9" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$2m</t>
         </is>
       </c>
       <c r="L9" s="15" t="inlineStr">
         <is>
-          <t>Esophageal SCC; Ovarian Ca; Gastric Ca</t>
+          <t>HER2+ Breast Ca; Gastric Ca; angiosarcoma</t>
         </is>
       </c>
       <c r="M9" s="15" t="inlineStr">
         <is>
-          <t>Commercial rights: ROW</t>
+          <t>All rights: Global</t>
         </is>
       </c>
       <c r="N9" s="15" t="inlineStr">
         <is>
-          <t>2025-07-08</t>
+          <t>2025-09-29</t>
         </is>
       </c>
       <c r="O9" s="17" t="inlineStr">
         <is>
-          <t>EU commercial rights to Gentili/Ewopharma. PDL1 mAb approved in CN/EU. CStone is HK-listed, capital-constrained with thin pipeline. EU royalty stream from sugemalimab is small but real. Worth approaching for broader balance sheet solution.</t>
+          <t>Global all rights to Gilead. US NDA filed. Hanmi is large KR pharma, generally well-capitalized. Small deal ($34.5M).</t>
         </is>
       </c>
     </row>
     <row r="10" ht="26.1" customHeight="1">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>RemeGen (荣昌生物)</t>
+          <t>CStone Pharmaceuticals (基石药业)</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
@@ -1393,22 +1393,22 @@
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>Vor Biopharma</t>
+          <t>Istituto Gentili</t>
         </is>
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>telitacicept (TACI | Fc-fusion)</t>
+          <t>sugemalimab (PDL1 | mAb)</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>Fusion Protein</t>
+          <t>mAb</t>
         </is>
       </c>
       <c r="F10" s="24" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Ph1</t>
         </is>
       </c>
       <c r="G10" s="16" t="inlineStr">
@@ -1418,49 +1418,49 @@
       </c>
       <c r="H10" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="I10" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="J10" s="16" t="inlineStr">
         <is>
-          <t>$4.2bn</t>
+          <t>$192m</t>
         </is>
       </c>
       <c r="K10" s="16" t="inlineStr">
         <is>
-          <t>$45m</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L10" s="15" t="inlineStr">
         <is>
-          <t>IgAvasculitis; IgA Nephropathy; idiopathic membranous nephropathy</t>
+          <t>Esophageal SCC; Ovarian Ca; Gastric Ca</t>
         </is>
       </c>
       <c r="M10" s="15" t="inlineStr">
         <is>
-          <t>All rights: US;EU;JP;ROW</t>
+          <t>Commercial rights: ROW</t>
         </is>
       </c>
       <c r="N10" s="15" t="inlineStr">
         <is>
-          <t>2025-06-26</t>
+          <t>2025-07-08</t>
         </is>
       </c>
       <c r="O10" s="17" t="inlineStr">
         <is>
-          <t>Potential FIC. Ex-CN all rights to Vor Biopharma. TACI fusion protein approved in CN for SLE, US/EU/JP all in Ph3, near-term ex-CN launch possible. $4.2bn total deal. RemeGen is HK-listed, cash-intensive global trials. Strong candidate for royalty monetization on ex-CN stream to fund retained pipeline.</t>
+          <t>EU commercial rights to Gentili/Ewopharma. PDL1 mAb approved in CN/EU. CStone is HK-listed, capital-constrained with thin pipeline. EU royalty stream from sugemalimab is small but real. Worth approaching for broader balance sheet solution.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="26.1" customHeight="1">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>3SBio (三生制药)</t>
+          <t>RemeGen (荣昌生物)</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
@@ -1470,17 +1470,17 @@
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>Pfizer</t>
+          <t>Vor Biopharma</t>
         </is>
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>SSGJ-707 (VEGF; PD1 | BsAb)</t>
+          <t>telitacicept (TACI | Fc-fusion)</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>mAb</t>
+          <t>Fusion Protein</t>
         </is>
       </c>
       <c r="F11" s="24" t="inlineStr">
@@ -1490,74 +1490,74 @@
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
           <t>Ph3</t>
         </is>
       </c>
-      <c r="H11" s="16" t="inlineStr">
+      <c r="I11" s="16" t="inlineStr">
         <is>
           <t>Ph3</t>
         </is>
       </c>
-      <c r="I11" s="16" t="inlineStr">
-        <is>
-          <t>Ph3</t>
-        </is>
-      </c>
       <c r="J11" s="16" t="inlineStr">
         <is>
-          <t>$6.2bn</t>
+          <t>$4.2bn</t>
         </is>
       </c>
       <c r="K11" s="16" t="inlineStr">
         <is>
-          <t>$1.2bn</t>
+          <t>$45m</t>
         </is>
       </c>
       <c r="L11" s="15" t="inlineStr">
         <is>
-          <t>NSCLC; Ovarian Ca; non-sq NSCLC</t>
+          <t>IgAvasculitis; IgA Nephropathy; idiopathic membranous nephropathy</t>
         </is>
       </c>
       <c r="M11" s="15" t="inlineStr">
         <is>
-          <t>All rights: HK/TW;US;EU;JP;ROW | R&amp;D rights(opt.): CN | Commercial rights(opt.): CN</t>
+          <t>All rights: US;EU;JP;ROW</t>
         </is>
       </c>
       <c r="N11" s="15" t="inlineStr">
         <is>
-          <t>2025-05-20</t>
+          <t>2025-06-26</t>
         </is>
       </c>
       <c r="O11" s="17" t="inlineStr">
         <is>
-          <t>Ex-CN all rights to Pfizer. PD1×VEGF BsAb in Ph3 globally, competitive but well-validated space. $6.2bn headline with $1.25bn upfront shows Pfizer conviction. 3SBio mid-cap, may consider royalty monetization.</t>
+          <t>Potential FIC. Ex-CN all rights to Vor Biopharma. TACI fusion protein approved in CN for SLE, US/EU/JP all in Ph3, near-term ex-CN launch possible. $4.2bn total deal. RemeGen is HK-listed, cash-intensive global trials. Strong candidate for royalty monetization on ex-CN stream to fund retained pipeline.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="26.1" customHeight="1">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>Nxera Pharma</t>
+          <t>3SBio (三生制药)</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>Viatris</t>
+          <t>Pfizer</t>
         </is>
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>cenerimod (S1PR1 | S1PR1modulator)</t>
+          <t>SSGJ-707 (VEGF; PD1 | BsAb)</t>
         </is>
       </c>
       <c r="E12" s="15" t="inlineStr">
         <is>
-          <t>Small Mol.</t>
+          <t>mAb</t>
         </is>
       </c>
       <c r="F12" s="24" t="inlineStr">
@@ -1582,39 +1582,39 @@
       </c>
       <c r="J12" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$6.2bn</t>
         </is>
       </c>
       <c r="K12" s="16" t="inlineStr">
         <is>
-          <t>$10m</t>
+          <t>$1.2bn</t>
         </is>
       </c>
       <c r="L12" s="15" t="inlineStr">
         <is>
-          <t>SLE; Lupus Nephritis</t>
+          <t>NSCLC; Ovarian Ca; non-sq NSCLC</t>
         </is>
       </c>
       <c r="M12" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: JP;ROW | Commercial rights: JP;ROW</t>
+          <t>All rights: HK/TW;US;EU;JP;ROW | R&amp;D rights(opt.): CN | Commercial rights(opt.): CN</t>
         </is>
       </c>
       <c r="N12" s="15" t="inlineStr">
         <is>
-          <t>2025-02-28</t>
+          <t>2025-05-20</t>
         </is>
       </c>
       <c r="O12" s="17" t="inlineStr">
         <is>
-          <t>JP/ROW R&amp;D + commercial to Viatris. S1P1 modulator in Ph3 for SLE. Nxera (fmr Sosei) is JP mid-cap GPCR specialist. Retained rights limited. Moderate RBF interest, Nxera has ongoing cash needs but deal economics may be thin.</t>
+          <t>Ex-CN all rights to Pfizer. PD1×VEGF BsAb in Ph3 globally, competitive but well-validated space. $6.2bn headline with $1.25bn upfront shows Pfizer conviction. 3SBio mid-cap, may consider royalty monetization.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="26.1" customHeight="1">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Stella Pharma</t>
+          <t>Nxera Pharma</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
@@ -1624,12 +1624,12 @@
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>TAE Life Sciences</t>
+          <t>Viatris</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>boron(10B)-falan (SLC7A5 | BNCT)</t>
+          <t>cenerimod (S1PR1 | S1PR1modulator)</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
@@ -1639,22 +1639,22 @@
       </c>
       <c r="F13" s="24" t="inlineStr">
         <is>
-          <t>Ph1/2</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="G13" s="16" t="inlineStr">
         <is>
-          <t>Ph2</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="H13" s="16" t="inlineStr">
         <is>
-          <t>Ph2</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="I13" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="J13" s="16" t="inlineStr">
@@ -1664,79 +1664,79 @@
       </c>
       <c r="K13" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$10m</t>
         </is>
       </c>
       <c r="L13" s="15" t="inlineStr">
         <is>
-          <t>meningioma; H&amp;N Cancer; brain Ca</t>
+          <t>SLE; Lupus Nephritis</t>
         </is>
       </c>
       <c r="M13" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: US;EU | Commercial rights: US;EU</t>
+          <t>R&amp;D rights: JP;ROW | Commercial rights: JP;ROW</t>
         </is>
       </c>
       <c r="N13" s="15" t="inlineStr">
         <is>
-          <t>2024-11-13</t>
+          <t>2025-02-28</t>
         </is>
       </c>
       <c r="O13" s="17" t="inlineStr">
         <is>
-          <t>Potential FIC. US/EU rights out-licensed. R&amp;D + commercial rights. JP; BNCT niche.</t>
+          <t>JP/ROW R&amp;D + commercial to Viatris. S1P1 modulator in Ph3 for SLE. Nxera (fmr Sosei) is JP mid-cap GPCR specialist. Retained rights limited. Moderate RBF interest, Nxera has ongoing cash needs but deal economics may be thin.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="26.1" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>Ensol Biosciences</t>
+          <t>Stella Pharma</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>Korea</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>Spine BioPharma</t>
+          <t>TAE Life Sciences</t>
         </is>
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>vicatertide (TGF-β1 | TGF-β1modulator)</t>
+          <t>boron(10B)-falan (SLC7A5 | BNCT)</t>
         </is>
       </c>
       <c r="E14" s="15" t="inlineStr">
         <is>
-          <t>Peptide</t>
+          <t>Small Mol.</t>
         </is>
       </c>
       <c r="F14" s="24" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Ph1/2</t>
         </is>
       </c>
       <c r="G14" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Ph2</t>
         </is>
       </c>
       <c r="H14" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Ph2</t>
         </is>
       </c>
       <c r="I14" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="J14" s="16" t="inlineStr">
         <is>
-          <t>$155m</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K14" s="16" t="inlineStr">
@@ -1746,64 +1746,64 @@
       </c>
       <c r="L14" s="15" t="inlineStr">
         <is>
-          <t>DDD; Low Back Pain</t>
+          <t>meningioma; H&amp;N Cancer; brain Ca</t>
         </is>
       </c>
       <c r="M14" s="15" t="inlineStr">
         <is>
-          <t>All rights: Global</t>
+          <t>R&amp;D rights: US;EU | Commercial rights: US;EU</t>
         </is>
       </c>
       <c r="N14" s="15" t="inlineStr">
         <is>
-          <t>2024-07-10</t>
+          <t>2024-11-13</t>
         </is>
       </c>
       <c r="O14" s="17" t="inlineStr">
         <is>
-          <t>Potential FIC. Global all rights out. TGF-b1 modulator for disc degeneration, niche orthopedic indication. KR biotech, small deal ($155M).</t>
+          <t>Potential FIC. US/EU rights out-licensed. R&amp;D + commercial rights. JP; BNCT niche.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="26.1" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>CStone Pharmaceuticals (基石药业)</t>
+          <t>Ensol Biosciences</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Korea</t>
         </is>
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>Ewopharma</t>
+          <t>Spine BioPharma</t>
         </is>
       </c>
       <c r="D15" s="15" t="inlineStr">
         <is>
-          <t>sugemalimab (PDL1 | mAb)</t>
+          <t>vicatertide (TGF-β1 | TGF-β1modulator)</t>
         </is>
       </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
-          <t>mAb</t>
+          <t>Peptide</t>
         </is>
       </c>
       <c r="F15" s="24" t="inlineStr">
         <is>
-          <t>Ph1</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="G15" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="H15" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="I15" s="16" t="inlineStr">
@@ -1813,64 +1813,64 @@
       </c>
       <c r="J15" s="16" t="inlineStr">
         <is>
+          <t>$155m</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K15" s="16" t="inlineStr">
-        <is>
-          <t>$51m</t>
-        </is>
-      </c>
       <c r="L15" s="15" t="inlineStr">
         <is>
-          <t>Esophageal SCC; Ovarian Ca; Gastric Ca</t>
+          <t>DDD; Low Back Pain</t>
         </is>
       </c>
       <c r="M15" s="15" t="inlineStr">
         <is>
-          <t>Commercial rights: ROW</t>
+          <t>All rights: Global</t>
         </is>
       </c>
       <c r="N15" s="15" t="inlineStr">
         <is>
-          <t>2024-05-27</t>
+          <t>2024-07-10</t>
         </is>
       </c>
       <c r="O15" s="17" t="inlineStr">
         <is>
-          <t>EU commercial rights to Gentili/Ewopharma.</t>
+          <t>Potential FIC. Global all rights out. TGF-b1 modulator for disc degeneration, niche orthopedic indication. KR biotech, small deal ($155M).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="26.1" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>Toray Industries</t>
+          <t>CStone Pharmaceuticals (基石药业)</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>Immunis</t>
+          <t>Ewopharma</t>
         </is>
       </c>
       <c r="D16" s="15" t="inlineStr">
         <is>
-          <t>nalfurafine (κ opioid receptor | κ opioid receptoragonist)</t>
+          <t>sugemalimab (PDL1 | mAb)</t>
         </is>
       </c>
       <c r="E16" s="15" t="inlineStr">
         <is>
-          <t>Small Mol.</t>
+          <t>mAb</t>
         </is>
       </c>
       <c r="F16" s="24" t="inlineStr">
         <is>
-          <t>Ph2</t>
+          <t>Ph1</t>
         </is>
       </c>
       <c r="G16" s="16" t="inlineStr">
@@ -1880,12 +1880,12 @@
       </c>
       <c r="H16" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="I16" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="J16" s="16" t="inlineStr">
@@ -1895,111 +1895,111 @@
       </c>
       <c r="K16" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$51m</t>
         </is>
       </c>
       <c r="L16" s="15" t="inlineStr">
         <is>
-          <t>Pruritus in CLD; liver disease; Uremic Pruritus</t>
+          <t>Esophageal SCC; Ovarian Ca; Gastric Ca</t>
         </is>
       </c>
       <c r="M16" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: JP | Commercial rights: JP</t>
+          <t>Commercial rights: ROW</t>
         </is>
       </c>
       <c r="N16" s="15" t="inlineStr">
         <is>
-          <t>2024-05-22</t>
+          <t>2024-05-27</t>
         </is>
       </c>
       <c r="O16" s="17" t="inlineStr">
         <is>
-          <t>Potential FIC. JP-only rights. R&amp;D + commercial rights. JP conglomerate.</t>
+          <t>EU commercial rights to Gentili/Ewopharma.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="26.1" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>Hengrui Medicine (恒瑞医药)</t>
+          <t>Toray Industries</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>Kailera (NewCo)</t>
+          <t>Immunis</t>
         </is>
       </c>
       <c r="D17" s="15" t="inlineStr">
         <is>
-          <t>HRS9531 (GLP-1R; GIPR | GIPRagonist/GLP-1Ragonist)</t>
+          <t>nalfurafine (κ opioid receptor | κ opioid receptoragonist)</t>
         </is>
       </c>
       <c r="E17" s="15" t="inlineStr">
         <is>
-          <t>Peptide</t>
+          <t>Small Mol.</t>
         </is>
       </c>
       <c r="F17" s="24" t="inlineStr">
         <is>
+          <t>Ph2</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
           <t>Ph3</t>
         </is>
       </c>
-      <c r="G17" s="16" t="inlineStr">
-        <is>
-          <t>NDA Filed</t>
-        </is>
-      </c>
-      <c r="H17" s="16" t="inlineStr">
-        <is>
-          <t>Preclnl</t>
-        </is>
-      </c>
       <c r="I17" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="J17" s="16" t="inlineStr">
         <is>
-          <t>$6.0bn</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K17" s="16" t="inlineStr">
         <is>
-          <t>$100m</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L17" s="15" t="inlineStr">
         <is>
-          <t>Diabetes; Obesity; ASCVD</t>
+          <t>Pruritus in CLD; liver disease; Uremic Pruritus</t>
         </is>
       </c>
       <c r="M17" s="15" t="inlineStr">
         <is>
-          <t>All rights: US;EU;JP;ROW</t>
+          <t>R&amp;D rights: JP | Commercial rights: JP</t>
         </is>
       </c>
       <c r="N17" s="15" t="inlineStr">
         <is>
-          <t>2024-05-16</t>
+          <t>2024-05-22</t>
         </is>
       </c>
       <c r="O17" s="17" t="inlineStr">
         <is>
-          <t>Ex-CN all rights to Kailera (NewCo). GLP-1R/GIPR dual agonist, CN NDA filed, US Ph3. $6bn deal but only $100M upfront, heavily milestone-loaded. Hengrui is large-cap, self-funded, unlikely to need RBF. However, Kailera as a NewCo licensee could be an interesting angle from the other side.</t>
+          <t>Potential FIC. JP-only rights. R&amp;D + commercial rights. JP conglomerate.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="26.1" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Hansoh Pharma (翰森制药)</t>
+          <t>Hengrui Medicine (恒瑞医药)</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
@@ -2009,17 +2009,17 @@
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>GSK</t>
+          <t>Kailera (NewCo)</t>
         </is>
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>risvutatug rezetecan (B7-H3 | anti-B7-H3ADC)</t>
+          <t>HRS9531 (GLP-1R; GIPR | GIPRagonist/GLP-1Ragonist)</t>
         </is>
       </c>
       <c r="E18" s="15" t="inlineStr">
         <is>
-          <t>ADC</t>
+          <t>Peptide</t>
         </is>
       </c>
       <c r="F18" s="24" t="inlineStr">
@@ -2029,32 +2029,32 @@
       </c>
       <c r="G18" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>NDA Filed</t>
         </is>
       </c>
       <c r="H18" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="I18" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="J18" s="16" t="inlineStr">
         <is>
-          <t>$1.7bn</t>
+          <t>$6.0bn</t>
         </is>
       </c>
       <c r="K18" s="16" t="inlineStr">
         <is>
-          <t>$185m</t>
+          <t>$100m</t>
         </is>
       </c>
       <c r="L18" s="15" t="inlineStr">
         <is>
-          <t>HNSCC; Gastric Ca; STS</t>
+          <t>Diabetes; Obesity; ASCVD</t>
         </is>
       </c>
       <c r="M18" s="15" t="inlineStr">
@@ -2064,19 +2064,19 @@
       </c>
       <c r="N18" s="15" t="inlineStr">
         <is>
-          <t>2023-12-20</t>
+          <t>2024-05-16</t>
         </is>
       </c>
       <c r="O18" s="17" t="inlineStr">
         <is>
-          <t>Ex-CN all rights to GSK. B7-H3 ADC in Ph3 globally. $1.7bn deal, $185M upfront. Hansoh profitable, low RBF need. But GSK validation of B7-H3 ADC space is notable.</t>
+          <t>Ex-CN all rights to Kailera (NewCo). GLP-1R/GIPR dual agonist, CN NDA filed, US Ph3. $6bn deal but only $100M upfront, heavily milestone-loaded. Hengrui is large-cap, self-funded, unlikely to need RBF. However, Kailera as a NewCo licensee could be an interesting angle from the other side.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="26.1" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Biokin Pharma (百利天恒)</t>
+          <t>Hansoh Pharma (翰森制药)</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
@@ -2086,12 +2086,12 @@
       </c>
       <c r="C19" s="15" t="inlineStr">
         <is>
-          <t>Bristol-Myers Squibb</t>
+          <t>GSK</t>
         </is>
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>BL-B01D1 (HER3; EGFR | ADC)</t>
+          <t>risvutatug rezetecan (B7-H3 | anti-B7-H3ADC)</t>
         </is>
       </c>
       <c r="E19" s="15" t="inlineStr">
@@ -2101,59 +2101,59 @@
       </c>
       <c r="F19" s="24" t="inlineStr">
         <is>
-          <t>Ph2/3</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="G19" s="16" t="inlineStr">
         <is>
-          <t>NDA Filed</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="H19" s="16" t="inlineStr">
         <is>
-          <t>Ph2/3</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="I19" s="16" t="inlineStr">
         <is>
-          <t>Ph2/3</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="J19" s="16" t="inlineStr">
         <is>
-          <t>$8.4bn</t>
+          <t>$1.7bn</t>
         </is>
       </c>
       <c r="K19" s="16" t="inlineStr">
         <is>
-          <t>$800m</t>
+          <t>$185m</t>
         </is>
       </c>
       <c r="L19" s="15" t="inlineStr">
         <is>
-          <t>Prostate Ca; Pancreatic Ca; Melanoma</t>
+          <t>HNSCC; Gastric Ca; STS</t>
         </is>
       </c>
       <c r="M19" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: US;EU;JP;ROW | Commercial rights: US;EU;JP;ROW</t>
+          <t>All rights: US;EU;JP;ROW</t>
         </is>
       </c>
       <c r="N19" s="15" t="inlineStr">
         <is>
-          <t>2023-12-12</t>
+          <t>2023-12-20</t>
         </is>
       </c>
       <c r="O19" s="17" t="inlineStr">
         <is>
-          <t>Potential FIC. Ex-CN R&amp;D + commercial to BMS. EGFR×HER3 bispecific ADC, $8.4bn headline is one of the largest China out-license deals ever. US/EU Ph2/3, CN NDA filed. Biokin is SH-listed mid-cap with limited other revenue, retains CN rights but needs capital to fund commercial launch. Strong RBF candidate for CN royalty stream or structured financing against BMS milestones.</t>
+          <t>Ex-CN all rights to GSK. B7-H3 ADC in Ph3 globally. $1.7bn deal, $185M upfront. Hansoh profitable, low RBF need. But GSK validation of B7-H3 ADC space is notable.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="26.1" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>Biotheus Inc (普米斯)</t>
+          <t>Biokin Pharma (百利天恒)</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
@@ -2163,99 +2163,99 @@
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>BioNTech</t>
+          <t>Bristol-Myers Squibb</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>PM8002 (VEGF-A; PDL1 | anti-PDL1×VEGF-ABsAb)</t>
+          <t>BL-B01D1 (HER3; EGFR | ADC)</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>mAb</t>
+          <t>ADC</t>
         </is>
       </c>
       <c r="F20" s="24" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Ph2/3</t>
         </is>
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>NDA Filed</t>
         </is>
       </c>
       <c r="H20" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Ph2/3</t>
         </is>
       </c>
       <c r="I20" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Ph2/3</t>
         </is>
       </c>
       <c r="J20" s="16" t="inlineStr">
         <is>
-          <t>$1.1bn</t>
+          <t>$8.4bn</t>
         </is>
       </c>
       <c r="K20" s="16" t="inlineStr">
         <is>
-          <t>$55m</t>
+          <t>$800m</t>
         </is>
       </c>
       <c r="L20" s="15" t="inlineStr">
         <is>
-          <t>SCLC; CRC; GBM</t>
+          <t>Prostate Ca; Pancreatic Ca; Melanoma</t>
         </is>
       </c>
       <c r="M20" s="15" t="inlineStr">
         <is>
-          <t>All rights: US;EU;JP;ROW</t>
+          <t>R&amp;D rights: US;EU;JP;ROW | Commercial rights: US;EU;JP;ROW</t>
         </is>
       </c>
       <c r="N20" s="15" t="inlineStr">
         <is>
-          <t>2023-11-06</t>
+          <t>2023-12-12</t>
         </is>
       </c>
       <c r="O20" s="17" t="inlineStr">
         <is>
-          <t>Potential FIC. Ex-CN all rights to BioNTech. PDL1×VEGF-A BsAb in Ph3 globally. Private company, capital-intensive, strong candidate for royalty financing. BioNTech partnership validates asset quality.</t>
+          <t>Potential FIC. Ex-CN R&amp;D + commercial to BMS. EGFR×HER3 bispecific ADC, $8.4bn headline is one of the largest China out-license deals ever. US/EU Ph2/3, CN NDA filed. Biokin is SH-listed mid-cap with limited other revenue, retains CN rights but needs capital to fund commercial launch. Strong RBF candidate for CN royalty stream or structured financing against BMS milestones.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="26.1" customHeight="1">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>Biotheus Inc (普米斯)</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>Merck &amp; Co.</t>
+          <t>BioNTech</t>
         </is>
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>patritumab deruxtecan (HER3 | ADC)</t>
+          <t>PM8002 (VEGF-A; PDL1 | anti-PDL1×VEGF-ABsAb)</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>ADC</t>
+          <t>mAb</t>
         </is>
       </c>
       <c r="F21" s="24" t="inlineStr">
         <is>
-          <t>NDA Filed</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="G21" s="16" t="inlineStr">
@@ -2275,32 +2275,32 @@
       </c>
       <c r="J21" s="16" t="inlineStr">
         <is>
-          <t>$22.0bn</t>
+          <t>$1.1bn</t>
         </is>
       </c>
       <c r="K21" s="16" t="inlineStr">
         <is>
-          <t>$4.0bn</t>
+          <t>$55m</t>
         </is>
       </c>
       <c r="L21" s="15" t="inlineStr">
         <is>
-          <t>Brain Metastases; Bladder Ca; NRG1fusion+ solid tumors</t>
+          <t>SCLC; CRC; GBM</t>
         </is>
       </c>
       <c r="M21" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: Global | Commercial rights: Global</t>
+          <t>All rights: US;EU;JP;ROW</t>
         </is>
       </c>
       <c r="N21" s="15" t="inlineStr">
         <is>
-          <t>2023-10-19</t>
+          <t>2023-11-06</t>
         </is>
       </c>
       <c r="O21" s="17" t="inlineStr">
         <is>
-          <t>Global R&amp;D + commercial to Merck. HER3 ADC, US NDA filed. Part of $22bn deal. Daiichi self-funded, no RBF angle.</t>
+          <t>Potential FIC. Ex-CN all rights to BioNTech. PDL1×VEGF-A BsAb in Ph3 globally. Private company, capital-intensive, strong candidate for royalty financing. BioNTech partnership validates asset quality.</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="D22" s="15" t="inlineStr">
         <is>
-          <t>ifinatamab deruxtecan (B7-H3 | anti-B7-H3ADC)</t>
+          <t>patritumab deruxtecan (HER3 | ADC)</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
@@ -2332,24 +2332,24 @@
       </c>
       <c r="F22" s="24" t="inlineStr">
         <is>
+          <t>NDA Filed</t>
+        </is>
+      </c>
+      <c r="G22" s="16" t="inlineStr">
+        <is>
           <t>Ph3</t>
         </is>
       </c>
-      <c r="G22" s="16" t="inlineStr">
+      <c r="H22" s="16" t="inlineStr">
         <is>
           <t>Ph3</t>
         </is>
       </c>
-      <c r="H22" s="16" t="inlineStr">
+      <c r="I22" s="16" t="inlineStr">
         <is>
           <t>Ph3</t>
         </is>
       </c>
-      <c r="I22" s="16" t="inlineStr">
-        <is>
-          <t>Ph3</t>
-        </is>
-      </c>
       <c r="J22" s="16" t="inlineStr">
         <is>
           <t>$22.0bn</t>
@@ -2362,7 +2362,7 @@
       </c>
       <c r="L22" s="15" t="inlineStr">
         <is>
-          <t>Esophageal adeno Ca; Esophageal Ca; non-sq NSCLC</t>
+          <t>Brain Metastases; Bladder Ca; NRG1fusion+ solid tumors</t>
         </is>
       </c>
       <c r="M22" s="15" t="inlineStr">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="O22" s="17" t="inlineStr">
         <is>
-          <t>Potential FIC. Global R&amp;D + commercial to Merck. B7-H3 ADC Ph3 globally. Part of $22bn mega-deal. No RBF need, large-cap JP pharma.</t>
+          <t>Global R&amp;D + commercial to Merck. HER3 ADC, US NDA filed. Part of $22bn deal. Daiichi self-funded, no RBF angle.</t>
         </is>
       </c>
     </row>
@@ -2399,7 +2399,7 @@
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
-          <t>raludotatug deruxtecan (CDH6 | ADC)</t>
+          <t>ifinatamab deruxtecan (B7-H3 | anti-B7-H3ADC)</t>
         </is>
       </c>
       <c r="E23" s="15" t="inlineStr">
@@ -2409,22 +2409,22 @@
       </c>
       <c r="F23" s="24" t="inlineStr">
         <is>
-          <t>Ph2/3</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="G23" s="16" t="inlineStr">
         <is>
-          <t>Ph2/3</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="H23" s="16" t="inlineStr">
         <is>
-          <t>Ph2/3</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="I23" s="16" t="inlineStr">
         <is>
-          <t>Ph2/3</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="J23" s="16" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="L23" s="15" t="inlineStr">
         <is>
-          <t>Esophageal Ca; Endometrial Ca; extrahepatic cholangiocarcinoma</t>
+          <t>Esophageal adeno Ca; Esophageal Ca; non-sq NSCLC</t>
         </is>
       </c>
       <c r="M23" s="15" t="inlineStr">
@@ -2454,29 +2454,29 @@
       </c>
       <c r="O23" s="17" t="inlineStr">
         <is>
-          <t>Global R&amp;D + commercial to Merck. CDH6 ADC, part of $22bn DaSi mega-deal. Daiichi Sankyo is large-cap JP, no RBF need.</t>
+          <t>Potential FIC. Global R&amp;D + commercial to Merck. B7-H3 ADC Ph3 globally. Part of $22bn mega-deal. No RBF need, large-cap JP pharma.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="26.1" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>DualityBio (映恩生物)</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>BioNTech</t>
+          <t>Merck &amp; Co.</t>
         </is>
       </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
-          <t>DB-1303 (HER2 | ADC)</t>
+          <t>raludotatug deruxtecan (CDH6 | ADC)</t>
         </is>
       </c>
       <c r="E24" s="15" t="inlineStr">
@@ -2486,59 +2486,59 @@
       </c>
       <c r="F24" s="24" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Ph2/3</t>
         </is>
       </c>
       <c r="G24" s="16" t="inlineStr">
         <is>
-          <t>NDA Filed</t>
+          <t>Ph2/3</t>
         </is>
       </c>
       <c r="H24" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Ph2/3</t>
         </is>
       </c>
       <c r="I24" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Ph2/3</t>
         </is>
       </c>
       <c r="J24" s="16" t="inlineStr">
         <is>
-          <t>$1.7bn</t>
+          <t>$22.0bn</t>
         </is>
       </c>
       <c r="K24" s="16" t="inlineStr">
         <is>
-          <t>$170m</t>
+          <t>$4.0bn</t>
         </is>
       </c>
       <c r="L24" s="15" t="inlineStr">
         <is>
-          <t>TNBC; HER2-low Breast Ca; HER2+ Breast Ca</t>
+          <t>Esophageal Ca; Endometrial Ca; extrahepatic cholangiocarcinoma</t>
         </is>
       </c>
       <c r="M24" s="15" t="inlineStr">
         <is>
-          <t>All rights: US;EU;JP;ROW</t>
+          <t>R&amp;D rights: Global | Commercial rights: Global</t>
         </is>
       </c>
       <c r="N24" s="15" t="inlineStr">
         <is>
-          <t>2023-04-03</t>
+          <t>2023-10-19</t>
         </is>
       </c>
       <c r="O24" s="17" t="inlineStr">
         <is>
-          <t>Ex-CN all rights to BioNTech. HER2 ADC in US/EU Ph3, CN NDA filed. $1.67bn deal. DualityBio is private with multiple ADC programs burning cash, potential candidate for royalty financing on BioNTech deal stream.</t>
+          <t>Global R&amp;D + commercial to Merck. CDH6 ADC, part of $22bn DaSi mega-deal. Daiichi Sankyo is large-cap JP, no RBF need.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="26.1" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>KYM Biosciences</t>
+          <t>DualityBio (映恩生物)</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
@@ -2548,12 +2548,12 @@
       </c>
       <c r="C25" s="15" t="inlineStr">
         <is>
-          <t>AstraZeneca</t>
+          <t>BioNTech</t>
         </is>
       </c>
       <c r="D25" s="15" t="inlineStr">
         <is>
-          <t>visonatatug (CLDN18.2 | anti-CLDN18.2ADC)</t>
+          <t>DB-1303 (HER2 | ADC)</t>
         </is>
       </c>
       <c r="E25" s="15" t="inlineStr">
@@ -2568,54 +2568,54 @@
       </c>
       <c r="G25" s="16" t="inlineStr">
         <is>
+          <t>NDA Filed</t>
+        </is>
+      </c>
+      <c r="H25" s="16" t="inlineStr">
+        <is>
           <t>Ph3</t>
         </is>
       </c>
-      <c r="H25" s="16" t="inlineStr">
-        <is>
-          <t>Ph3</t>
-        </is>
-      </c>
       <c r="I25" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="J25" s="16" t="inlineStr">
         <is>
-          <t>$1.2bn</t>
+          <t>$1.7bn</t>
         </is>
       </c>
       <c r="K25" s="16" t="inlineStr">
         <is>
-          <t>$63m</t>
+          <t>$170m</t>
         </is>
       </c>
       <c r="L25" s="15" t="inlineStr">
         <is>
-          <t>PDAC; Pancreatic Ca; Esophageal Ca</t>
+          <t>TNBC; HER2-low Breast Ca; HER2+ Breast Ca</t>
         </is>
       </c>
       <c r="M25" s="15" t="inlineStr">
         <is>
-          <t>All rights: Global</t>
+          <t>All rights: US;EU;JP;ROW</t>
         </is>
       </c>
       <c r="N25" s="15" t="inlineStr">
         <is>
-          <t>2023-02-23</t>
+          <t>2023-04-03</t>
         </is>
       </c>
       <c r="O25" s="17" t="inlineStr">
         <is>
-          <t>Global all rights out-licensed. CLDN18.2 ADC to AZ, Ph3 globally. $1.2bn deal. JV structure (Keymed/Lepu) complicates, need to understand economics split. AZ validation strong but JV may limit clean royalty structuring.</t>
+          <t>Ex-CN all rights to BioNTech. HER2 ADC in US/EU Ph3, CN NDA filed. $1.67bn deal. DualityBio is private with multiple ADC programs burning cash, potential candidate for royalty financing on BioNTech deal stream.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="26.1" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>Akeso (康方生物)</t>
+          <t>KYM Biosciences</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
@@ -2625,27 +2625,27 @@
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>Summit Therapeutics</t>
+          <t>AstraZeneca</t>
         </is>
       </c>
       <c r="D26" s="15" t="inlineStr">
         <is>
-          <t>ivonescimab (VEGF-A; PD1 | anti-PD1×VEGF-ABsAb)</t>
+          <t>visonatatug (CLDN18.2 | anti-CLDN18.2ADC)</t>
         </is>
       </c>
       <c r="E26" s="15" t="inlineStr">
         <is>
-          <t>mAb</t>
+          <t>ADC</t>
         </is>
       </c>
       <c r="F26" s="24" t="inlineStr">
         <is>
-          <t>NDA Filed</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="G26" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="H26" s="16" t="inlineStr">
@@ -2660,59 +2660,59 @@
       </c>
       <c r="J26" s="16" t="inlineStr">
         <is>
-          <t>$5.0bn</t>
+          <t>$1.2bn</t>
         </is>
       </c>
       <c r="K26" s="16" t="inlineStr">
         <is>
-          <t>$500m</t>
+          <t>$63m</t>
         </is>
       </c>
       <c r="L26" s="15" t="inlineStr">
         <is>
-          <t>NSCLC; MIBC; GEJ Ca</t>
+          <t>PDAC; Pancreatic Ca; Esophageal Ca</t>
         </is>
       </c>
       <c r="M26" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: US;EU;JP;ROW | Commercial rights: US;EU;JP;ROW</t>
+          <t>All rights: Global</t>
         </is>
       </c>
       <c r="N26" s="15" t="inlineStr">
         <is>
-          <t>2022-12-06</t>
+          <t>2023-02-23</t>
         </is>
       </c>
       <c r="O26" s="17" t="inlineStr">
         <is>
-          <t>Potential FIC. Ex-CN R&amp;D + commercial to Summit. US NDA filed, CN approved. Near-term US revenue. Akeso growing but capital needs moderate.</t>
+          <t>Global all rights out-licensed. CLDN18.2 ADC to AZ, Ph3 globally. $1.2bn deal. JV structure (Keymed/Lepu) complicates, need to understand economics split. AZ validation strong but JV may limit clean royalty structuring.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="26.1" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>inno.N</t>
+          <t>Akeso (康方生物)</t>
         </is>
       </c>
       <c r="B27" s="15" t="inlineStr">
         <is>
-          <t>Korea</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>Sebela Pharmaceuticals</t>
+          <t>Summit Therapeutics</t>
         </is>
       </c>
       <c r="D27" s="15" t="inlineStr">
         <is>
-          <t>tegoprazan (proton pump | P-CAB)</t>
+          <t>ivonescimab (VEGF-A; PD1 | anti-PD1×VEGF-ABsAb)</t>
         </is>
       </c>
       <c r="E27" s="15" t="inlineStr">
         <is>
-          <t>Small Mol.</t>
+          <t>mAb</t>
         </is>
       </c>
       <c r="F27" s="24" t="inlineStr">
@@ -2727,64 +2727,64 @@
       </c>
       <c r="H27" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="I27" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="J27" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$5.0bn</t>
         </is>
       </c>
       <c r="K27" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$500m</t>
         </is>
       </c>
       <c r="L27" s="15" t="inlineStr">
         <is>
-          <t>NERD; peptic ulcer bleeding; Peptic Ulcer</t>
+          <t>NSCLC; MIBC; GEJ Ca</t>
         </is>
       </c>
       <c r="M27" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: US | Commercial rights: US</t>
+          <t>R&amp;D rights: US;EU;JP;ROW | Commercial rights: US;EU;JP;ROW</t>
         </is>
       </c>
       <c r="N27" s="15" t="inlineStr">
         <is>
-          <t>2022-10-19</t>
+          <t>2022-12-06</t>
         </is>
       </c>
       <c r="O27" s="17" t="inlineStr">
         <is>
-          <t>US R&amp;D + commercial to Sebela. P-CAB for GERD, US NDA filed, CN approved. KR mid-pharma, generally funded. Niche GI</t>
+          <t>Potential FIC. Ex-CN R&amp;D + commercial to Summit. US NDA filed, CN approved. Near-term US revenue. Akeso growing but capital needs moderate.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="26.1" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>Takeda Pharmaceuticals</t>
+          <t>inno.N</t>
         </is>
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Korea</t>
         </is>
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>Puma Biotechnology</t>
+          <t>Sebela Pharmaceuticals</t>
         </is>
       </c>
       <c r="D28" s="15" t="inlineStr">
         <is>
-          <t>alisertib (Aurora A | Aurora Ainh.)</t>
+          <t>tegoprazan (proton pump | P-CAB)</t>
         </is>
       </c>
       <c r="E28" s="15" t="inlineStr">
@@ -2794,59 +2794,59 @@
       </c>
       <c r="F28" s="24" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>NDA Filed</t>
         </is>
       </c>
       <c r="G28" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="H28" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="I28" s="16" t="inlineStr">
         <is>
-          <t>Ph1</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="J28" s="16" t="inlineStr">
         <is>
-          <t>$294m</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K28" s="16" t="inlineStr">
         <is>
-          <t>$7m</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L28" s="15" t="inlineStr">
         <is>
-          <t>ALCL; HNSCC; rhabdomyosarcoma</t>
+          <t>NERD; peptic ulcer bleeding; Peptic Ulcer</t>
         </is>
       </c>
       <c r="M28" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: Global | Commercial rights: Global</t>
+          <t>R&amp;D rights: US | Commercial rights: US</t>
         </is>
       </c>
       <c r="N28" s="15" t="inlineStr">
         <is>
-          <t>2022-09-20</t>
+          <t>2022-10-19</t>
         </is>
       </c>
       <c r="O28" s="17" t="inlineStr">
         <is>
-          <t>Potential FIC. Global R&amp;D + commercial to Puma. Aurora A inhibitor Ph3. Takeda is MNC, no RBF need.</t>
+          <t>US R&amp;D + commercial to Sebela. P-CAB for GERD, US NDA filed, CN approved. KR mid-pharma, generally funded. Niche GI</t>
         </is>
       </c>
     </row>
     <row r="29" ht="26.1" customHeight="1">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>Astellas Pharma</t>
+          <t>Takeda Pharmaceuticals</t>
         </is>
       </c>
       <c r="B29" s="15" t="inlineStr">
@@ -2856,12 +2856,12 @@
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>Sling Therapeutics</t>
+          <t>Puma Biotechnology</t>
         </is>
       </c>
       <c r="D29" s="15" t="inlineStr">
         <is>
-          <t>linsitinib (InsR; IGF-1R | InsRinh./IGF-1Rinh.)</t>
+          <t>alisertib (Aurora A | Aurora Ainh.)</t>
         </is>
       </c>
       <c r="E29" s="15" t="inlineStr">
@@ -2876,7 +2876,7 @@
       </c>
       <c r="G29" s="16" t="inlineStr">
         <is>
-          <t>IND Filed</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="H29" s="16" t="inlineStr">
@@ -2886,64 +2886,64 @@
       </c>
       <c r="I29" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Ph1</t>
         </is>
       </c>
       <c r="J29" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$294m</t>
         </is>
       </c>
       <c r="K29" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$7m</t>
         </is>
       </c>
       <c r="L29" s="15" t="inlineStr">
         <is>
-          <t>GIST; Ewing sarcoma; Breast Ca</t>
+          <t>ALCL; HNSCC; rhabdomyosarcoma</t>
         </is>
       </c>
       <c r="M29" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: US;EU</t>
+          <t>R&amp;D rights: Global | Commercial rights: Global</t>
         </is>
       </c>
       <c r="N29" s="15" t="inlineStr">
         <is>
-          <t>2022-06-13</t>
+          <t>2022-09-20</t>
         </is>
       </c>
       <c r="O29" s="17" t="inlineStr">
         <is>
-          <t>US/EU R&amp;D rights only. JP MNC, self-funded, no RBF need.</t>
+          <t>Potential FIC. Global R&amp;D + commercial to Puma. Aurora A inhibitor Ph3. Takeda is MNC, no RBF need.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="26.1" customHeight="1">
       <c r="A30" s="15" t="inlineStr">
         <is>
-          <t>Kelun-Biotech (科伦博泰)</t>
+          <t>Astellas Pharma</t>
         </is>
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C30" s="15" t="inlineStr">
         <is>
-          <t>Merck &amp; Co.</t>
+          <t>Sling Therapeutics</t>
         </is>
       </c>
       <c r="D30" s="15" t="inlineStr">
         <is>
-          <t>sacituzumab tirumotecan (TROP2 | ADC)</t>
+          <t>linsitinib (InsR; IGF-1R | InsRinh./IGF-1Rinh.)</t>
         </is>
       </c>
       <c r="E30" s="15" t="inlineStr">
         <is>
-          <t>ADC</t>
+          <t>Small Mol.</t>
         </is>
       </c>
       <c r="F30" s="24" t="inlineStr">
@@ -2953,7 +2953,7 @@
       </c>
       <c r="G30" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>IND Filed</t>
         </is>
       </c>
       <c r="H30" s="16" t="inlineStr">
@@ -2963,64 +2963,64 @@
       </c>
       <c r="I30" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="J30" s="16" t="inlineStr">
         <is>
-          <t>$1.4bn</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K30" s="16" t="inlineStr">
         <is>
-          <t>$47m</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L30" s="15" t="inlineStr">
         <is>
-          <t>NPC; MIBC; Cervical Ca</t>
+          <t>GIST; Ewing sarcoma; Breast Ca</t>
         </is>
       </c>
       <c r="M30" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: US;EU;JP;ROW | Commercial rights: US;EU;JP;ROW</t>
+          <t>R&amp;D rights: US;EU</t>
         </is>
       </c>
       <c r="N30" s="15" t="inlineStr">
         <is>
-          <t>2022-05-16</t>
+          <t>2022-06-13</t>
         </is>
       </c>
       <c r="O30" s="17" t="inlineStr">
         <is>
-          <t>Ex-CN R&amp;D + commercial to Merck. TROP2 ADC approved in CN, US/EU/JP Ph3. $1.4bn deal. Kelun-Biotech is HK-listed, parent-backed. Moderate RBF interest, Merck deal royalty stream is real but parent Kelun Pharma provides capital cushion.</t>
+          <t>US/EU R&amp;D rights only. JP MNC, self-funded, no RBF need.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="26.1" customHeight="1">
       <c r="A31" s="15" t="inlineStr">
         <is>
-          <t>EA Pharma</t>
+          <t>Kelun-Biotech (科伦博泰)</t>
         </is>
       </c>
       <c r="B31" s="15" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>Pathalys Pharma</t>
+          <t>Merck &amp; Co.</t>
         </is>
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
-          <t>upacicalcet (CaSR | CaSRmodulator)</t>
+          <t>sacituzumab tirumotecan (TROP2 | ADC)</t>
         </is>
       </c>
       <c r="E31" s="15" t="inlineStr">
         <is>
-          <t>Small Mol.</t>
+          <t>ADC</t>
         </is>
       </c>
       <c r="F31" s="24" t="inlineStr">
@@ -3030,7 +3030,7 @@
       </c>
       <c r="G31" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="H31" s="16" t="inlineStr">
@@ -3040,44 +3040,44 @@
       </c>
       <c r="I31" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="J31" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$1.4bn</t>
         </is>
       </c>
       <c r="K31" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$47m</t>
         </is>
       </c>
       <c r="L31" s="15" t="inlineStr">
         <is>
-          <t>Secondary HPT in CKD; ESRD; CKD Anemia</t>
+          <t>NPC; MIBC; Cervical Ca</t>
         </is>
       </c>
       <c r="M31" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: US;EU;ROW | Commercial rights: US;EU;ROW</t>
+          <t>R&amp;D rights: US;EU;JP;ROW | Commercial rights: US;EU;JP;ROW</t>
         </is>
       </c>
       <c r="N31" s="15" t="inlineStr">
         <is>
-          <t>2022-03-01</t>
+          <t>2022-05-16</t>
         </is>
       </c>
       <c r="O31" s="17" t="inlineStr">
         <is>
-          <t>Potential FIC. US/EU/ROW R&amp;D + commercial to Pathalys. CaSR modulator, JP approved, US/EU Ph3. JP mid-cap, Eisai subsidiary.</t>
+          <t>Ex-CN R&amp;D + commercial to Merck. TROP2 ADC approved in CN, US/EU/JP Ph3. $1.4bn deal. Kelun-Biotech is HK-listed, parent-backed. Moderate RBF interest, Merck deal royalty stream is real but parent Kelun Pharma provides capital cushion.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="26.1" customHeight="1">
       <c r="A32" s="15" t="inlineStr">
         <is>
-          <t>Nxera Pharma</t>
+          <t>EA Pharma</t>
         </is>
       </c>
       <c r="B32" s="15" t="inlineStr">
@@ -3087,12 +3087,12 @@
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>Neurocrine Biosciences</t>
+          <t>Pathalys Pharma</t>
         </is>
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
-          <t>direclidine (M4 receptor | M4 receptororthostericagonist)</t>
+          <t>upacicalcet (CaSR | CaSRmodulator)</t>
         </is>
       </c>
       <c r="E32" s="15" t="inlineStr">
@@ -3117,64 +3117,64 @@
       </c>
       <c r="I32" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="J32" s="16" t="inlineStr">
         <is>
-          <t>$2.7bn</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K32" s="16" t="inlineStr">
         <is>
-          <t>$100m</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L32" s="15" t="inlineStr">
         <is>
-          <t>Bipolar I; Alzheimer's Disease; manic episodes</t>
+          <t>Secondary HPT in CKD; ESRD; CKD Anemia</t>
         </is>
       </c>
       <c r="M32" s="15" t="inlineStr">
         <is>
-          <t>Commercial rights: Global | R&amp;D rights: Global</t>
+          <t>R&amp;D rights: US;EU;ROW | Commercial rights: US;EU;ROW</t>
         </is>
       </c>
       <c r="N32" s="15" t="inlineStr">
         <is>
-          <t>2021-11-22</t>
+          <t>2022-03-01</t>
         </is>
       </c>
       <c r="O32" s="17" t="inlineStr">
         <is>
-          <t>Potential FIC. Global R&amp;D + commercial to Neurocrine. M4 agonist Ph3 for schizophrenia, large CNS TAM. $2.7bn deal. Nxera could consider royalty monetization to fund GPCR pipeline, but JP corporate culture may resist.</t>
+          <t>Potential FIC. US/EU/ROW R&amp;D + commercial to Pathalys. CaSR modulator, JP approved, US/EU Ph3. JP mid-cap, Eisai subsidiary.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="26.1" customHeight="1">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>RemeGen (荣昌生物)</t>
+          <t>Nxera Pharma</t>
         </is>
       </c>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>Seagen</t>
+          <t>Neurocrine Biosciences</t>
         </is>
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
-          <t>disitamab vedotin (HER2 | ADC)</t>
+          <t>direclidine (M4 receptor | M4 receptororthostericagonist)</t>
         </is>
       </c>
       <c r="E33" s="15" t="inlineStr">
         <is>
-          <t>ADC</t>
+          <t>Small Mol.</t>
         </is>
       </c>
       <c r="F33" s="24" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="G33" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="H33" s="16" t="inlineStr">
@@ -3194,44 +3194,44 @@
       </c>
       <c r="I33" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="J33" s="16" t="inlineStr">
         <is>
-          <t>$2.6bn</t>
+          <t>$2.7bn</t>
         </is>
       </c>
       <c r="K33" s="16" t="inlineStr">
         <is>
-          <t>$200m</t>
+          <t>$100m</t>
         </is>
       </c>
       <c r="L33" s="15" t="inlineStr">
         <is>
-          <t>vaginal Ca; HER2-low Breast Ca; Solid tumors</t>
+          <t>Bipolar I; Alzheimer's Disease; manic episodes</t>
         </is>
       </c>
       <c r="M33" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: US;EU;JP;ROW | Commercial rights: US;EU;JP;ROW</t>
+          <t>Commercial rights: Global | R&amp;D rights: Global</t>
         </is>
       </c>
       <c r="N33" s="15" t="inlineStr">
         <is>
-          <t>2021-08-09</t>
+          <t>2021-11-22</t>
         </is>
       </c>
       <c r="O33" s="17" t="inlineStr">
         <is>
-          <t>Ex-CN R&amp;D + commercial to Seagen (now Pfizer). HER2 ADC approved in CN, US/EU/JP Ph3. $2.6bn deal, $200M upfront. Two approved assets (this + telitacicept) give RemeGen near-term royalty streams. Capital-intensive global expansion.</t>
+          <t>Potential FIC. Global R&amp;D + commercial to Neurocrine. M4 agonist Ph3 for schizophrenia, large CNS TAM. $2.7bn deal. Nxera could consider royalty monetization to fund GPCR pipeline, but JP corporate culture may resist.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="26.1" customHeight="1">
       <c r="A34" s="15" t="inlineStr">
         <is>
-          <t>Allist Pharmaceuticals (艾力斯)</t>
+          <t>RemeGen (荣昌生物)</t>
         </is>
       </c>
       <c r="B34" s="15" t="inlineStr">
@@ -3241,17 +3241,17 @@
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>ArriVent Biopharma (NewCo)</t>
+          <t>Seagen</t>
         </is>
       </c>
       <c r="D34" s="15" t="inlineStr">
         <is>
-          <t>furmonertinib (EGFR T790M; EGFR exon 20; HER2 exon 20 | EGFR T790Minh.)</t>
+          <t>disitamab vedotin (HER2 | ADC)</t>
         </is>
       </c>
       <c r="E34" s="15" t="inlineStr">
         <is>
-          <t>Small Mol.</t>
+          <t>ADC</t>
         </is>
       </c>
       <c r="F34" s="24" t="inlineStr">
@@ -3276,54 +3276,54 @@
       </c>
       <c r="J34" s="16" t="inlineStr">
         <is>
-          <t>$805m</t>
+          <t>$2.6bn</t>
         </is>
       </c>
       <c r="K34" s="16" t="inlineStr">
         <is>
-          <t>$40m</t>
+          <t>$200m</t>
         </is>
       </c>
       <c r="L34" s="15" t="inlineStr">
         <is>
-          <t>Breast Ca; malignant pleural effusion; Brain Metastases</t>
+          <t>vaginal Ca; HER2-low Breast Ca; Solid tumors</t>
         </is>
       </c>
       <c r="M34" s="15" t="inlineStr">
         <is>
-          <t>All rights: US;EU;JP;ROW</t>
+          <t>R&amp;D rights: US;EU;JP;ROW | Commercial rights: US;EU;JP;ROW</t>
         </is>
       </c>
       <c r="N34" s="15" t="inlineStr">
         <is>
-          <t>2021-06-30</t>
+          <t>2021-08-09</t>
         </is>
       </c>
       <c r="O34" s="17" t="inlineStr">
         <is>
-          <t>Ex-CN all rights to ArriVent (NewCo). 3rd-gen EGFR TKI approved in CN, US/EU/JP Ph3. $805M deal. Allist is SH-listed, growing CN revenue from furmonertinib. Global trial costs are significant. Moderate RBF interest, ArriVent royalty stream develops as US approval approaches.</t>
+          <t>Ex-CN R&amp;D + commercial to Seagen (now Pfizer). HER2 ADC approved in CN, US/EU/JP Ph3. $2.6bn deal, $200M upfront. Two approved assets (this + telitacicept) give RemeGen near-term royalty streams. Capital-intensive global expansion.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="26.1" customHeight="1">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t>Fuji Yakuhin</t>
+          <t>Allist Pharmaceuticals (艾力斯)</t>
         </is>
       </c>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>Fortress Biotech</t>
+          <t>ArriVent Biopharma (NewCo)</t>
         </is>
       </c>
       <c r="D35" s="15" t="inlineStr">
         <is>
-          <t>dotinurad (URAT1 | URAT1inh.)</t>
+          <t>furmonertinib (EGFR T790M; EGFR exon 20; HER2 exon 20 | EGFR T790Minh.)</t>
         </is>
       </c>
       <c r="E35" s="15" t="inlineStr">
@@ -3348,44 +3348,44 @@
       </c>
       <c r="I35" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="J35" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$805m</t>
         </is>
       </c>
       <c r="K35" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$40m</t>
         </is>
       </c>
       <c r="L35" s="15" t="inlineStr">
         <is>
-          <t>Gout; CKD; Heart Failure</t>
+          <t>Breast Ca; malignant pleural effusion; Brain Metastases</t>
         </is>
       </c>
       <c r="M35" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: US;EU | Commercial rights: US;EU</t>
+          <t>All rights: US;EU;JP;ROW</t>
         </is>
       </c>
       <c r="N35" s="15" t="inlineStr">
         <is>
-          <t>2021-05-10</t>
+          <t>2021-06-30</t>
         </is>
       </c>
       <c r="O35" s="17" t="inlineStr">
         <is>
-          <t>US/EU R&amp;D + commercial to Fortress. URAT1 inhibitor, JP approved, US/EU Ph3. JP mid-cap.</t>
+          <t>Ex-CN all rights to ArriVent (NewCo). 3rd-gen EGFR TKI approved in CN, US/EU/JP Ph3. $805M deal. Allist is SH-listed, growing CN revenue from furmonertinib. Global trial costs are significant. Moderate RBF interest, ArriVent royalty stream develops as US approval approaches.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="26.1" customHeight="1">
       <c r="A36" s="15" t="inlineStr">
         <is>
-          <t>Tanabe Pharma Corporation</t>
+          <t>Fuji Yakuhin</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
@@ -3395,12 +3395,12 @@
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>Mineralys Therapeutics</t>
+          <t>Fortress Biotech</t>
         </is>
       </c>
       <c r="D36" s="15" t="inlineStr">
         <is>
-          <t>lorundrostat (ALDOS | ALDOSinh.)</t>
+          <t>dotinurad (URAT1 | URAT1inh.)</t>
         </is>
       </c>
       <c r="E36" s="15" t="inlineStr">
@@ -3410,12 +3410,12 @@
       </c>
       <c r="F36" s="24" t="inlineStr">
         <is>
-          <t>NDA Filed</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="G36" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="H36" s="16" t="inlineStr">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="I36" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="J36" s="16" t="inlineStr">
@@ -3440,44 +3440,44 @@
       </c>
       <c r="L36" s="15" t="inlineStr">
         <is>
-          <t>OSA; Hypertension</t>
+          <t>Gout; CKD; Heart Failure</t>
         </is>
       </c>
       <c r="M36" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: Global</t>
+          <t>R&amp;D rights: US;EU | Commercial rights: US;EU</t>
         </is>
       </c>
       <c r="N36" s="15" t="inlineStr">
         <is>
-          <t>2021-04-06</t>
+          <t>2021-05-10</t>
         </is>
       </c>
       <c r="O36" s="17" t="inlineStr">
         <is>
-          <t>Global R&amp;D to Mineralys. Aldosterone synthase inhibitor, US NDA filed. Mitsubishi subsidiary, parent funded. Low RBF need.</t>
+          <t>US/EU R&amp;D + commercial to Fortress. URAT1 inhibitor, JP approved, US/EU Ph3. JP mid-cap.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="26.1" customHeight="1">
       <c r="A37" s="15" t="inlineStr">
         <is>
-          <t>SK Biopharma</t>
+          <t>Tanabe Pharma Corporation</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>Korea</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>Aerial BioPharma</t>
+          <t>Mineralys Therapeutics</t>
         </is>
       </c>
       <c r="D37" s="15" t="inlineStr">
         <is>
-          <t>solriamfetol (TAAR1; NET; DAT; 5-HT1A receptor | 5-HT1A receptoragonist;)</t>
+          <t>lorundrostat (ALDOS | ALDOSinh.)</t>
         </is>
       </c>
       <c r="E37" s="15" t="inlineStr">
@@ -3487,17 +3487,17 @@
       </c>
       <c r="F37" s="24" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>NDA Filed</t>
         </is>
       </c>
       <c r="G37" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="H37" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="I37" s="16" t="inlineStr">
@@ -3517,44 +3517,44 @@
       </c>
       <c r="L37" s="15" t="inlineStr">
         <is>
-          <t>Narcolepsy-EDS; binge eating disorder; shift-work sleep--wake disorder</t>
+          <t>OSA; Hypertension</t>
         </is>
       </c>
       <c r="M37" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: US;EU;ROW | Commercial rights: US;EU;ROW</t>
+          <t>R&amp;D rights: Global</t>
         </is>
       </c>
       <c r="N37" s="15" t="inlineStr">
         <is>
-          <t>2021-01-01</t>
+          <t>2021-04-06</t>
         </is>
       </c>
       <c r="O37" s="17" t="inlineStr">
         <is>
-          <t>Potential FIC. US/EU/ROW R&amp;D + commercial to Aerial. Multi-target CNS drug, approved in US/EU/CN. SK Group subsidiary, well funded.</t>
+          <t>Global R&amp;D to Mineralys. Aldosterone synthase inhibitor, US NDA filed. Mitsubishi subsidiary, parent funded. Low RBF need.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="26.1" customHeight="1">
       <c r="A38" s="15" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo</t>
+          <t>SK Biopharma</t>
         </is>
       </c>
       <c r="B38" s="15" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Korea</t>
         </is>
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>Rain</t>
+          <t>Aerial BioPharma</t>
         </is>
       </c>
       <c r="D38" s="15" t="inlineStr">
         <is>
-          <t>milademetan (MDM2 | MDM2inh.)</t>
+          <t>solriamfetol (TAAR1; NET; DAT; 5-HT1A receptor | 5-HT1A receptoragonist;)</t>
         </is>
       </c>
       <c r="E38" s="15" t="inlineStr">
@@ -3564,22 +3564,22 @@
       </c>
       <c r="F38" s="24" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="G38" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="H38" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="I38" s="16" t="inlineStr">
         <is>
-          <t>Ph1</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="J38" s="16" t="inlineStr">
@@ -3594,22 +3594,22 @@
       </c>
       <c r="L38" s="15" t="inlineStr">
         <is>
-          <t>Multiple Myeloma; Lymphoma; HR+ Breast Ca</t>
+          <t>Narcolepsy-EDS; binge eating disorder; shift-work sleep--wake disorder</t>
         </is>
       </c>
       <c r="M38" s="15" t="inlineStr">
         <is>
-          <t>Commercial rights: Global | R&amp;D rights: Global</t>
+          <t>R&amp;D rights: US;EU;ROW | Commercial rights: US;EU;ROW</t>
         </is>
       </c>
       <c r="N38" s="15" t="inlineStr">
         <is>
-          <t>2020-09-02</t>
+          <t>2021-01-01</t>
         </is>
       </c>
       <c r="O38" s="17" t="inlineStr">
         <is>
-          <t>Potential FIC. Global R&amp;D + commercial to Rain. MDM2 inhibitor Ph3. No RBF need.</t>
+          <t>Potential FIC. US/EU/ROW R&amp;D + commercial to Aerial. Multi-target CNS drug, approved in US/EU/CN. SK Group subsidiary, well funded.</t>
         </is>
       </c>
     </row>
@@ -3626,74 +3626,74 @@
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>AstraZeneca</t>
+          <t>Rain</t>
         </is>
       </c>
       <c r="D39" s="15" t="inlineStr">
         <is>
-          <t>dato-DXd (TROP2 | ADC)</t>
+          <t>milademetan (MDM2 | MDM2inh.)</t>
         </is>
       </c>
       <c r="E39" s="15" t="inlineStr">
         <is>
-          <t>ADC</t>
+          <t>Small Mol.</t>
         </is>
       </c>
       <c r="F39" s="24" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="G39" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="H39" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Ph3</t>
         </is>
       </c>
       <c r="I39" s="16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Ph1</t>
         </is>
       </c>
       <c r="J39" s="16" t="inlineStr">
         <is>
-          <t>$6.0bn</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K39" s="16" t="inlineStr">
         <is>
-          <t>$1.0bn</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L39" s="15" t="inlineStr">
         <is>
-          <t>TNBC; non-sq NSCLC; NSCLC</t>
+          <t>Multiple Myeloma; Lymphoma; HR+ Breast Ca</t>
         </is>
       </c>
       <c r="M39" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: Global | Commercial rights: Global</t>
+          <t>Commercial rights: Global | R&amp;D rights: Global</t>
         </is>
       </c>
       <c r="N39" s="15" t="inlineStr">
         <is>
-          <t>2020-07-27</t>
+          <t>2020-09-02</t>
         </is>
       </c>
       <c r="O39" s="17" t="inlineStr">
         <is>
-          <t>Global R&amp;D + commercial to AZ. TROP2 ADC, approved in US/EU/JP/CN. $6bn deal. Daiichi self-funded.</t>
+          <t>Potential FIC. Global R&amp;D + commercial to Rain. MDM2 inhibitor Ph3. No RBF need.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="26.1" customHeight="1">
       <c r="A40" s="15" t="inlineStr">
         <is>
-          <t>Takeda Pharmaceuticals</t>
+          <t>Daiichi Sankyo</t>
         </is>
       </c>
       <c r="B40" s="15" t="inlineStr">
@@ -3703,89 +3703,89 @@
       </c>
       <c r="C40" s="15" t="inlineStr">
         <is>
-          <t>Neurocrine Biosciences</t>
+          <t>AstraZeneca</t>
         </is>
       </c>
       <c r="D40" s="15" t="inlineStr">
         <is>
-          <t>osavampator (AMPA receptor | AMPA receptorPAMmodulator)</t>
+          <t>dato-DXd (TROP2 | ADC)</t>
         </is>
       </c>
       <c r="E40" s="15" t="inlineStr">
         <is>
-          <t>Small Mol.</t>
+          <t>ADC</t>
         </is>
       </c>
       <c r="F40" s="24" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="G40" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="H40" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="I40" s="16" t="inlineStr">
         <is>
-          <t>Preclnl</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="J40" s="16" t="inlineStr">
         <is>
-          <t>$2.0bn</t>
+          <t>$6.0bn</t>
         </is>
       </c>
       <c r="K40" s="16" t="inlineStr">
         <is>
-          <t>$120m</t>
+          <t>$1.0bn</t>
         </is>
       </c>
       <c r="L40" s="15" t="inlineStr">
         <is>
-          <t>MDD; TRD; Depression</t>
+          <t>TNBC; non-sq NSCLC; NSCLC</t>
         </is>
       </c>
       <c r="M40" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights: CN;HK/TW;US;EU;ROW | Commercial rights: CN;HK/TW;US;EU;ROW</t>
+          <t>R&amp;D rights: Global | Commercial rights: Global</t>
         </is>
       </c>
       <c r="N40" s="15" t="inlineStr">
         <is>
-          <t>2020-06-16</t>
+          <t>2020-07-27</t>
         </is>
       </c>
       <c r="O40" s="17" t="inlineStr">
         <is>
-          <t>Potential FIC. Global R&amp;D + commercial to Neurocrine. AMPA PAM for MDD, novel CNS mechanism. $2bn deal. Takeda MNC, no RBF need.</t>
+          <t>Global R&amp;D + commercial to AZ. TROP2 ADC, approved in US/EU/JP/CN. $6bn deal. Daiichi self-funded.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="26.1" customHeight="1">
       <c r="A41" s="15" t="inlineStr">
         <is>
-          <t>Denovo Biopharma (索元生物)</t>
+          <t>Takeda Pharmaceuticals</t>
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C41" s="15" t="inlineStr">
         <is>
-          <t>Rumpus Therapeutics</t>
+          <t>Neurocrine Biosciences</t>
         </is>
       </c>
       <c r="D41" s="15" t="inlineStr">
         <is>
-          <t>enzastaurin (PKCβ | PKCβinh.)</t>
+          <t>osavampator (AMPA receptor | AMPA receptorPAMmodulator)</t>
         </is>
       </c>
       <c r="E41" s="15" t="inlineStr">
@@ -3800,122 +3800,199 @@
       </c>
       <c r="G41" s="16" t="inlineStr">
         <is>
+          <t>Preclnl</t>
+        </is>
+      </c>
+      <c r="H41" s="16" t="inlineStr">
+        <is>
           <t>Ph3</t>
         </is>
       </c>
-      <c r="H41" s="16" t="inlineStr">
-        <is>
-          <t>Ph3</t>
-        </is>
-      </c>
       <c r="I41" s="16" t="inlineStr">
         <is>
-          <t>Ph3</t>
+          <t>Preclnl</t>
         </is>
       </c>
       <c r="J41" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$2.0bn</t>
         </is>
       </c>
       <c r="K41" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$120m</t>
         </is>
       </c>
       <c r="L41" s="15" t="inlineStr">
         <is>
-          <t>FL; lymphocytic leukemia; Prostate Ca</t>
+          <t>MDD; TRD; Depression</t>
         </is>
       </c>
       <c r="M41" s="15" t="inlineStr">
         <is>
-          <t>R&amp;D rights(opt.): Global | Commercial rights(opt.): Global</t>
+          <t>R&amp;D rights: CN;HK/TW;US;EU;ROW | Commercial rights: CN;HK/TW;US;EU;ROW</t>
         </is>
       </c>
       <c r="N41" s="15" t="inlineStr">
         <is>
-          <t>2020-01-21</t>
+          <t>2020-06-16</t>
         </is>
       </c>
       <c r="O41" s="17" t="inlineStr">
         <is>
-          <t>Ex-CN R&amp;D + commercial (option) to Rumpus. PKCb inhibitor Ph3, biomarker-guided drug rescue model. Denovo is SH-listed, moderate cash. Novel model but commercial path uncertain. Moderate RBF interest.</t>
+          <t>Potential FIC. Global R&amp;D + commercial to Neurocrine. AMPA PAM for MDD, novel CNS mechanism. $2bn deal. Takeda MNC, no RBF need.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="26.1" customHeight="1">
       <c r="A42" s="15" t="inlineStr">
         <is>
+          <t>Denovo Biopharma (索元生物)</t>
+        </is>
+      </c>
+      <c r="B42" s="15" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="inlineStr">
+        <is>
+          <t>Rumpus Therapeutics</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
+        <is>
+          <t>enzastaurin (PKCβ | PKCβinh.)</t>
+        </is>
+      </c>
+      <c r="E42" s="15" t="inlineStr">
+        <is>
+          <t>Small Mol.</t>
+        </is>
+      </c>
+      <c r="F42" s="24" t="inlineStr">
+        <is>
+          <t>Ph3</t>
+        </is>
+      </c>
+      <c r="G42" s="16" t="inlineStr">
+        <is>
+          <t>Ph3</t>
+        </is>
+      </c>
+      <c r="H42" s="16" t="inlineStr">
+        <is>
+          <t>Ph3</t>
+        </is>
+      </c>
+      <c r="I42" s="16" t="inlineStr">
+        <is>
+          <t>Ph3</t>
+        </is>
+      </c>
+      <c r="J42" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K42" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L42" s="15" t="inlineStr">
+        <is>
+          <t>FL; lymphocytic leukemia; Prostate Ca</t>
+        </is>
+      </c>
+      <c r="M42" s="15" t="inlineStr">
+        <is>
+          <t>R&amp;D rights(opt.): Global | Commercial rights(opt.): Global</t>
+        </is>
+      </c>
+      <c r="N42" s="15" t="inlineStr">
+        <is>
+          <t>2020-01-21</t>
+        </is>
+      </c>
+      <c r="O42" s="17" t="inlineStr">
+        <is>
+          <t>Ex-CN R&amp;D + commercial (option) to Rumpus. PKCb inhibitor Ph3, biomarker-guided drug rescue model. Denovo is SH-listed, moderate cash. Novel model but commercial path uncertain. Moderate RBF interest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="26.1" customHeight="1">
+      <c r="A43" s="15" t="inlineStr">
+        <is>
           <t>Chugai Pharmaceutical</t>
         </is>
       </c>
-      <c r="B42" s="15" t="inlineStr">
+      <c r="B43" s="15" t="inlineStr">
         <is>
           <t>Japan</t>
         </is>
       </c>
-      <c r="C42" s="15" t="inlineStr">
+      <c r="C43" s="15" t="inlineStr">
         <is>
           <t>Verastem</t>
         </is>
       </c>
-      <c r="D42" s="15" t="inlineStr">
+      <c r="D43" s="15" t="inlineStr">
         <is>
           <t>avutometinib (ARAF; MEK1; MEK2; CRAF; BRAF | BRAFinh.)</t>
         </is>
       </c>
-      <c r="E42" s="15" t="inlineStr">
+      <c r="E43" s="15" t="inlineStr">
         <is>
           <t>Small Mol.</t>
         </is>
       </c>
-      <c r="F42" s="24" t="inlineStr">
+      <c r="F43" s="24" t="inlineStr">
         <is>
           <t>NDA Filed</t>
         </is>
       </c>
-      <c r="G42" s="16" t="inlineStr">
-        <is>
-          <t>Preclnl</t>
-        </is>
-      </c>
-      <c r="H42" s="16" t="inlineStr">
+      <c r="G43" s="16" t="inlineStr">
+        <is>
+          <t>Preclnl</t>
+        </is>
+      </c>
+      <c r="H43" s="16" t="inlineStr">
         <is>
           <t>Ph3</t>
         </is>
       </c>
-      <c r="I42" s="16" t="inlineStr">
+      <c r="I43" s="16" t="inlineStr">
         <is>
           <t>Ph3</t>
         </is>
       </c>
-      <c r="J42" s="16" t="inlineStr">
+      <c r="J43" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K42" s="16" t="inlineStr">
+      <c r="K43" s="16" t="inlineStr">
         <is>
           <t>$3m</t>
         </is>
       </c>
-      <c r="L42" s="15" t="inlineStr">
+      <c r="L43" s="15" t="inlineStr">
         <is>
           <t>Lung Adenocarcinoma; Gastric Ca; Endometrial Ca</t>
         </is>
       </c>
-      <c r="M42" s="15" t="inlineStr">
+      <c r="M43" s="15" t="inlineStr">
         <is>
           <t>R&amp;D rights: Global | Commercial rights: Global</t>
         </is>
       </c>
-      <c r="N42" s="15" t="inlineStr">
+      <c r="N43" s="15" t="inlineStr">
         <is>
           <t>2020-01-08</t>
         </is>
       </c>
-      <c r="O42" s="17" t="inlineStr">
+      <c r="O43" s="17" t="inlineStr">
         <is>
           <t>Potential FIC. Global R&amp;D + commercial to Verastem. MEK/RAF inhibitor, US NDA filed. Chugai is Roche subsidiary, no RBF need.</t>
         </is>

</xml_diff>